<commit_message>
Admin panel refactor: dynamic questions, restructured layout and fix text clipping
</commit_message>
<xml_diff>
--- a/public/NUEVO TEST DE ENEAGRAMA COMPLETO.xlsx
+++ b/public/NUEVO TEST DE ENEAGRAMA COMPLETO.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d054766ea3ab6770/Escritorio/Eneagrama/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAE9D6A-145A-4148-B2EF-2CB970919128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{0310297B-343C-47CE-AFF3-35FA3C55CE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AADFF047-5A59-4524-B2CE-C2F85543E70D}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{32DE2995-2421-4BC0-8390-3482C1C7896A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{32DE2995-2421-4BC0-8390-3482C1C7896A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Eneagrama Largo" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eneagrama Largo'!$A$1:$E$136</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,17 +30,16 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="205">
   <si>
     <t>E1</t>
   </si>
@@ -478,13 +480,190 @@
   </si>
   <si>
     <t>Busco que las relaciones se mantengan en paz.</t>
+  </si>
+  <si>
+    <t>Cuando algo no sale como esperaba, me resulta difícil dejarlo pasar porque sigo pensando cómo debería haberse hecho.</t>
+  </si>
+  <si>
+    <t>Tiendo a controlarme para actuar de la manera que considero correcta, incluso cuando me gustaría reaccionar distinto</t>
+  </si>
+  <si>
+    <t>Cambio</t>
+  </si>
+  <si>
+    <t>Suelo tomarme muy en serio mis deberes y compromisos, incluso cuando eso me genera presión interna.</t>
+  </si>
+  <si>
+    <t>Me siento especialmente bien cuando puedo ayudar o ser útil para alguien cercano.</t>
+  </si>
+  <si>
+    <t>Cuando alguien cercano está mal, siento casi automáticamente el impulso de cuidarlo o acompañarlo.</t>
+  </si>
+  <si>
+    <t>Suelo notar con facilidad lo que las personas necesitan emocionalmente y siento ganas de responder a ello.</t>
+  </si>
+  <si>
+    <t>Necesito sentir cercanía y cariño en mis relaciones para sentirme realmente tranquilo.</t>
+  </si>
+  <si>
+    <t>Disfruto sentir que aporto bienestar a las personas que quiero, porque eso me hace sentir valioso para ellas.</t>
+  </si>
+  <si>
+    <t>Me gusta sentir que avanzo, logro cosas y obtengo buenos resultados, porque eso me hace sentir que voy por buen camino.</t>
+  </si>
+  <si>
+    <t>Cuando me propongo una meta, pongo mucha energía en alcanzarla y me cuesta soltarla hasta lograrla.</t>
+  </si>
+  <si>
+    <t>Tiendo a mantenerme activo y enfocado en lo que quiero lograr, incluso cuando eso me mantiene siempre ocupado.</t>
+  </si>
+  <si>
+    <t>Puedo adaptarme con facilidad a distintas situaciones para que las cosas funcionen bien o salgan adelante.</t>
+  </si>
+  <si>
+    <t>Cuando algo no sale bien, me esfuerzo rápido por corregirlo y seguir adelante sin quedarme demasiado en el problema.</t>
+  </si>
+  <si>
+    <t>Me resulta importante aprovechar bien el tiempo y seguir avanzando hacia algo</t>
+  </si>
+  <si>
+    <t>Disfruto ver resultados concretos de mi esfuerzo, porque eso confirma que voy bien</t>
+  </si>
+  <si>
+    <t>Suelo vivir mis emociones con mucha intensidad y me cuesta ignorarlas o dejarlas pasar.</t>
+  </si>
+  <si>
+    <t>Me afecta profundamente lo que me pasa por dentro, incluso cuando otros no lo notan.</t>
+  </si>
+  <si>
+    <t>Puedo pasar mucho tiempo reflexionando sobre mis sentimientos para entenderlos.</t>
+  </si>
+  <si>
+    <t>Valoro mucho la autenticidad y expresar lo que realmente siento, aunque a veces me haga sentir vulnerable.</t>
+  </si>
+  <si>
+    <t>Las experiencias emocionales intensas suelen tener mucho significado para mí</t>
+  </si>
+  <si>
+    <t>Mi estado de ánimo puede cambiar fácilmente según lo que esté viviendo por dentro.</t>
+  </si>
+  <si>
+    <t>Me conmueve profundamente la belleza, el arte o los momentos que siento significativos.</t>
+  </si>
+  <si>
+    <t>Necesito sentir conexión emocional profunda para sentirme realmente bien.</t>
+  </si>
+  <si>
+    <t>Me importa ser fiel a lo que soy y a lo que siento por dentro, incluso cuando eso me hace sentir diferente.</t>
+  </si>
+  <si>
+    <t>Me gusta comprender las cosas a fondo antes de involucrarme o participar</t>
+  </si>
+  <si>
+    <t>Necesito momentos de soledad para recuperar energía y sentirme bien conmigo mismo.</t>
+  </si>
+  <si>
+    <t>Prefiero analizar bien las cosas antes de actuar.</t>
+  </si>
+  <si>
+    <t>Me interesa aprender, investigar y entender cómo funcionan las cosas en profundidad.</t>
+  </si>
+  <si>
+    <t>Valoro mucho mi independencia y mi espacio personal.</t>
+  </si>
+  <si>
+    <t>Me siento más seguro cuando entiendo bien lo que está pasando.</t>
+  </si>
+  <si>
+    <t>Prefiero pocas relaciones profundas y tranquilas antes que muchas relaciones superficiales.</t>
+  </si>
+  <si>
+    <t>Me siento mejor cuando tengo claridad mental sobre lo que está pasando a mi alrededor.</t>
+  </si>
+  <si>
+    <t>Me siento mucho más tranquilo cuando tengo claridad y seguridad sobre lo que podría pasar.</t>
+  </si>
+  <si>
+    <t>A veces dudo bastante antes de actuar porque pienso en distintas posibilidades.</t>
+  </si>
+  <si>
+    <t>Para mí es muy importante sentir que puedo confiar en las personas y en las situaciones.</t>
+  </si>
+  <si>
+    <t>Me tranquiliza sentir apoyo y respaldo cuando tengo que tomar decisiones importantes.</t>
+  </si>
+  <si>
+    <t>A veces pienso demasiado las cosas antes de decidir, tratando de prever lo que podría pasar.</t>
+  </si>
+  <si>
+    <t>Cuando asumo un compromiso, suelo tomarlo muy en serio.</t>
+  </si>
+  <si>
+    <t>Cuando confío en alguien, suelo mantenerme muy leal a esa persona.</t>
+  </si>
+  <si>
+    <t>Suelo buscar señales o información que me ayuden a sentirme seguro.</t>
+  </si>
+  <si>
+    <t>En situaciones nuevas, suelo observar primero hasta sentir que el ambiente es seguro.</t>
+  </si>
+  <si>
+    <t>Me siento mejor cuando sé que cuento con protección, apoyo o guía.</t>
+  </si>
+  <si>
+    <t>Suelo decir lo que pienso de forma directa, incluso si puede incomodar.</t>
+  </si>
+  <si>
+    <t>Prefiero tomar el mando antes que quedarme en segundo plano cuando algo es importante.</t>
+  </si>
+  <si>
+    <t>Valoro la fortaleza, la determinación y la capacidad de enfrentar las cosas de frente.</t>
+  </si>
+  <si>
+    <t>Siento la necesidad de proteger a las personas que quiero cuando percibo que algo las amenaza.</t>
+  </si>
+  <si>
+    <t>Prefiero actuar con decisión antes que quedarme mucho tiempo dudando.</t>
+  </si>
+  <si>
+    <t>Tiendo a enfrentar los problemas de frente en lugar de evitarlos.</t>
+  </si>
+  <si>
+    <t>Me gusta sentir que tengo el control de mi vida y de mis decisiones.</t>
+  </si>
+  <si>
+    <t>Respeto a las personas que son firmes, claras y no se dejan dominar.</t>
+  </si>
+  <si>
+    <t>Suelo adaptarme para que las cosas fluyan sin generar problemas.</t>
+  </si>
+  <si>
+    <t>Busco que las relaciones se mantengan en paz y sin tensiones.</t>
+  </si>
+  <si>
+    <t>Disfruto especialmente los momentos simples y tranquilos.</t>
+  </si>
+  <si>
+    <t>Suelo ver distintos puntos de vista en una misma situación antes de tomar posición.</t>
+  </si>
+  <si>
+    <t>Prefiero ambientes serenos antes que ambientes muy intensos o conflictivos.</t>
+  </si>
+  <si>
+    <t>Cuando hay conflicto, intento que las cosas vuelvan a estar bien entre todos.</t>
+  </si>
+  <si>
+    <t>Procuro que todo esté en calma y sin tensiones.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -500,13 +679,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -519,8 +705,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -543,20 +735,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -567,71 +765,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -642,15 +793,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13FB371B-D9F3-4571-BE01-BD05C6206802}" name="Tabla1" displayName="Tabla1" ref="C1:C136" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{74D48089-3E34-4AF8-A6FE-0B75B5C81CD4}" name="Preguntas" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -969,1516 +1111,2183 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42BAC113-3527-413A-8D1B-3B44CD1B33E9}">
-  <dimension ref="A1:C136"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEDE1B6D-1479-42CC-A67D-1530C449213C}">
+  <dimension ref="A1:F136"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.8984375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="90.69921875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="90.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="110.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2">
+      <c r="E1" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2">
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2">
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="2">
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="2">
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="1">
+        <v>5</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="2">
+      <c r="E6" s="8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="1">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="2">
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="1">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="2">
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="1">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="2">
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="1">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="2">
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="1">
+        <v>10</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="2">
+      <c r="E11" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="1">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="2">
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="1">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="2">
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="1">
+        <v>13</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="2">
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="1">
+        <v>14</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="2">
+      <c r="E15" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="1">
+        <v>15</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="2">
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="2">
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="1">
+        <v>2</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="2">
+      <c r="E18" s="7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="1">
+        <v>3</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="2">
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="1">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="2">
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="1">
+        <v>5</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2">
+      <c r="E21" s="7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="1">
+        <v>6</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="2">
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="1">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="2">
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="1">
+        <v>8</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="2">
+      <c r="E24" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="1">
+        <v>9</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="2">
+      <c r="E25" s="7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="1">
+        <v>10</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="2">
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="1">
+        <v>11</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="2">
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="1">
+        <v>12</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="2">
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="1">
+        <v>13</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="2">
+      <c r="E29" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="1">
+        <v>14</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="2">
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="1">
+        <v>15</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="2">
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="1">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="2">
+      <c r="E32" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="1">
+        <v>2</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="2">
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="1">
+        <v>3</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="2">
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="1">
+        <v>4</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="2">
+      <c r="E35" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="1">
+        <v>5</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="2">
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="1">
+        <v>6</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="2">
+      <c r="E37" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="1">
+        <v>7</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="2">
+      <c r="E38" s="5"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="1">
+        <v>8</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="2">
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="1">
+        <v>9</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="2">
+      <c r="E40" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="1">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="2">
+      <c r="E41" s="5"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="1">
+        <v>11</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" s="2">
+      <c r="E42" s="7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="1">
+        <v>12</v>
+      </c>
+      <c r="D43" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" s="2">
+      <c r="E43" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="1">
+        <v>13</v>
+      </c>
+      <c r="D44" s="7" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" s="2">
+      <c r="E44" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="1">
+        <v>14</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" s="2">
+      <c r="E45" s="5"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="1">
+        <v>15</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" s="2">
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="1">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="2">
+      <c r="E47" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="1">
+        <v>2</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" s="2">
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
         <v>48</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="1">
+        <v>3</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" s="2">
+      <c r="E49" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="1">
+        <v>4</v>
+      </c>
+      <c r="D50" s="7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" s="2">
+      <c r="E50" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="1">
+        <v>5</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" s="2">
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="1">
+        <v>6</v>
+      </c>
+      <c r="D52" s="7" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" s="2">
+      <c r="E52" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="1">
+        <v>7</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" s="2">
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="1">
+        <v>8</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" s="2">
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
         <v>54</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="1">
+        <v>9</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" s="2">
+      <c r="E55" s="7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
         <v>55</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="1">
+        <v>10</v>
+      </c>
+      <c r="D56" s="7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" s="2">
+      <c r="E56" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
         <v>56</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="1">
+        <v>11</v>
+      </c>
+      <c r="D57" s="7" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" s="2">
+      <c r="E57" s="7" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
         <v>57</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="C58" s="1">
+        <v>12</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" s="2">
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="1">
+        <v>13</v>
+      </c>
+      <c r="D59" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" s="2">
+      <c r="E59" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="1">
+        <v>14</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" s="2">
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="1">
+        <v>15</v>
+      </c>
+      <c r="D61" s="7" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" s="2">
+      <c r="E61" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
         <v>61</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="1">
+        <v>1</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" s="2">
+      <c r="E62" s="7" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
         <v>62</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C63" s="4" t="s">
+      <c r="C63" s="1">
+        <v>2</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" s="2">
+      <c r="E63" s="5"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
         <v>63</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="C64" s="1">
+        <v>3</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" s="2">
+      <c r="E64" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
         <v>64</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C65" s="1">
+        <v>4</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" s="2">
+      <c r="E65" s="5"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
         <v>65</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="C66" s="1">
+        <v>5</v>
+      </c>
+      <c r="D66" s="7" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" s="2">
+      <c r="E66" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
         <v>66</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C67" s="1">
+        <v>6</v>
+      </c>
+      <c r="D67" s="7" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" s="2">
+      <c r="E67" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
         <v>67</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="1">
+        <v>7</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" s="2">
+      <c r="E68" s="5"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
         <v>68</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C69" s="4" t="s">
+      <c r="C69" s="1">
+        <v>8</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" s="2">
+      <c r="E69" s="5"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
         <v>69</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C70" s="4" t="s">
+      <c r="C70" s="1">
+        <v>9</v>
+      </c>
+      <c r="D70" s="7" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="71" spans="1:3">
-      <c r="A71" s="2">
+      <c r="E70" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
         <v>70</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="C71" s="1">
+        <v>10</v>
+      </c>
+      <c r="D71" s="7" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="72" spans="1:3">
-      <c r="A72" s="2">
+      <c r="E71" s="7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
         <v>71</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="C72" s="1">
+        <v>11</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="73" spans="1:3">
-      <c r="A73" s="2">
+      <c r="E72" s="5"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
         <v>72</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C73" s="4" t="s">
+      <c r="C73" s="1">
+        <v>12</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="74" spans="1:3">
-      <c r="A74" s="2">
+      <c r="E73" s="5"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
         <v>73</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C74" s="4" t="s">
+      <c r="C74" s="1">
+        <v>13</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" s="2">
+      <c r="E74" s="7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
         <v>74</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="C75" s="1">
+        <v>14</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76" s="2">
+      <c r="E75" s="5"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
         <v>75</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C76" s="1">
+        <v>15</v>
+      </c>
+      <c r="D76" s="7" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="77" spans="1:3">
-      <c r="A77" s="2">
+      <c r="E76" s="7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
         <v>76</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="1">
+        <v>1</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="78" spans="1:3">
-      <c r="A78" s="2">
+      <c r="E77" s="2"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
         <v>77</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="1">
+        <v>2</v>
+      </c>
+      <c r="D78" s="7" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="79" spans="1:3">
-      <c r="A79" s="2">
+      <c r="E78" s="7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
         <v>78</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C79" s="1">
+        <v>3</v>
+      </c>
+      <c r="D79" s="7" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="80" spans="1:3">
-      <c r="A80" s="2">
+      <c r="E79" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
         <v>79</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="C80" s="1">
+        <v>4</v>
+      </c>
+      <c r="D80" s="7" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="81" spans="1:3">
-      <c r="A81" s="2">
+      <c r="E80" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
         <v>80</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="1">
+        <v>5</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82" s="2">
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
         <v>81</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="C82" s="1">
+        <v>6</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="83" spans="1:3">
-      <c r="A83" s="2">
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
         <v>82</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="1">
+        <v>7</v>
+      </c>
+      <c r="D83" s="7" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="84" spans="1:3">
-      <c r="A84" s="2">
+      <c r="E83" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
         <v>83</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="1">
+        <v>8</v>
+      </c>
+      <c r="D84" s="7" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85" s="2">
+      <c r="E84" s="7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
         <v>84</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C85" s="4" t="s">
+      <c r="C85" s="1">
+        <v>9</v>
+      </c>
+      <c r="D85" s="7" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="86" spans="1:3">
-      <c r="A86" s="2">
+      <c r="E85" s="7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
         <v>85</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C86" s="4" t="s">
+      <c r="C86" s="1">
+        <v>10</v>
+      </c>
+      <c r="D86" s="7" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="87" spans="1:3">
-      <c r="A87" s="2">
+      <c r="E86" s="7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
         <v>86</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="1">
+        <v>11</v>
+      </c>
+      <c r="D87" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
-      <c r="A88" s="2">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
         <v>87</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C88" s="4" t="s">
+      <c r="C88" s="1">
+        <v>12</v>
+      </c>
+      <c r="D88" s="7" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="89" spans="1:3">
-      <c r="A89" s="2">
+      <c r="E88" s="7" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
         <v>88</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" s="1">
+        <v>13</v>
+      </c>
+      <c r="D89" s="7" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="90" spans="1:3">
-      <c r="A90" s="2">
+      <c r="E89" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
         <v>89</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C90" s="4" t="s">
+      <c r="C90" s="1">
+        <v>14</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="91" spans="1:3">
-      <c r="A91" s="2">
+      <c r="E90" s="2"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
         <v>90</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="B91" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="C91" s="1">
+        <v>15</v>
+      </c>
+      <c r="D91" s="7" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="92" spans="1:3">
-      <c r="A92" s="2">
+      <c r="E91" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
         <v>91</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="B92" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="1">
+        <v>1</v>
+      </c>
+      <c r="D92" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="93" spans="1:3">
-      <c r="A93" s="2">
+      <c r="E92" s="5"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
         <v>92</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B93" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C93" s="4" t="s">
+      <c r="C93" s="1">
+        <v>2</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" s="2">
+      <c r="E93" s="5"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
         <v>93</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C94" s="4" t="s">
+      <c r="C94" s="1">
+        <v>3</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="95" spans="1:3">
-      <c r="A95" s="2">
+      <c r="E94" s="5"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
         <v>94</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B95" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="C95" s="1">
+        <v>4</v>
+      </c>
+      <c r="D95" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="96" spans="1:3">
-      <c r="A96" s="2">
+      <c r="E95" s="5"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
         <v>95</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C96" s="4" t="s">
+      <c r="C96" s="1">
+        <v>5</v>
+      </c>
+      <c r="D96" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="97" spans="1:3">
-      <c r="A97" s="2">
+      <c r="E96" s="5"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
         <v>96</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="1">
+        <v>6</v>
+      </c>
+      <c r="D97" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="98" spans="1:3">
-      <c r="A98" s="2">
+      <c r="E97" s="5"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
         <v>97</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C98" s="1">
+        <v>7</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99" s="2">
+      <c r="E98" s="5"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
         <v>98</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C99" s="1">
+        <v>8</v>
+      </c>
+      <c r="D99" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="100" spans="1:3">
-      <c r="A100" s="2">
+      <c r="E99" s="5"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
         <v>99</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C100" s="4" t="s">
+      <c r="C100" s="1">
+        <v>9</v>
+      </c>
+      <c r="D100" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="101" spans="1:3">
-      <c r="A101" s="2">
+      <c r="E100" s="5"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
         <v>100</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C101" s="1">
+        <v>10</v>
+      </c>
+      <c r="D101" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="102" spans="1:3">
-      <c r="A102" s="2">
+      <c r="E101" s="5"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
         <v>101</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C102" s="1">
+        <v>11</v>
+      </c>
+      <c r="D102" s="2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="103" spans="1:3">
-      <c r="A103" s="2">
+      <c r="E102" s="5"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
         <v>102</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C103" s="1">
+        <v>12</v>
+      </c>
+      <c r="D103" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="104" spans="1:3">
-      <c r="A104" s="2">
+      <c r="E103" s="5"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
         <v>103</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B104" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C104" s="4" t="s">
+      <c r="C104" s="1">
+        <v>13</v>
+      </c>
+      <c r="D104" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="105" spans="1:3">
-      <c r="A105" s="2">
+      <c r="E104" s="5"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
         <v>104</v>
       </c>
-      <c r="B105" s="2" t="s">
+      <c r="B105" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C105" s="4" t="s">
+      <c r="C105" s="1">
+        <v>14</v>
+      </c>
+      <c r="D105" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="106" spans="1:3">
-      <c r="A106" s="2">
+      <c r="E105" s="5"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
         <v>105</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="B106" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C106" s="4" t="s">
+      <c r="C106" s="1">
+        <v>15</v>
+      </c>
+      <c r="D106" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="107" spans="1:3">
-      <c r="A107" s="2">
+      <c r="E106" s="5"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
         <v>106</v>
       </c>
-      <c r="B107" s="2" t="s">
+      <c r="B107" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C107" s="4" t="s">
+      <c r="C107" s="1">
+        <v>1</v>
+      </c>
+      <c r="D107" s="7" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="108" spans="1:3">
-      <c r="A108" s="2">
+      <c r="E107" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
         <v>107</v>
       </c>
-      <c r="B108" s="2" t="s">
+      <c r="B108" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C108" s="4" t="s">
+      <c r="C108" s="1">
+        <v>2</v>
+      </c>
+      <c r="D108" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="109" spans="1:3">
-      <c r="A109" s="2">
+      <c r="E108" s="5"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
         <v>108</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="B109" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C109" s="4" t="s">
+      <c r="C109" s="1">
+        <v>3</v>
+      </c>
+      <c r="D109" s="7" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="110" spans="1:3">
-      <c r="A110" s="2">
+      <c r="E109" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
         <v>109</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="B110" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C110" s="4" t="s">
+      <c r="C110" s="1">
+        <v>4</v>
+      </c>
+      <c r="D110" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="111" spans="1:3">
-      <c r="A111" s="2">
+      <c r="E110" s="5"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
         <v>110</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="B111" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C111" s="4" t="s">
+      <c r="C111" s="1">
+        <v>5</v>
+      </c>
+      <c r="D111" s="7" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="112" spans="1:3">
-      <c r="A112" s="2">
+      <c r="E111" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
         <v>111</v>
       </c>
-      <c r="B112" s="2" t="s">
+      <c r="B112" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C112" s="4" t="s">
+      <c r="C112" s="1">
+        <v>6</v>
+      </c>
+      <c r="D112" s="2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="113" spans="1:3">
-      <c r="A113" s="2">
+      <c r="E112" s="5"/>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
         <v>112</v>
       </c>
-      <c r="B113" s="2" t="s">
+      <c r="B113" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C113" s="4" t="s">
+      <c r="C113" s="1">
+        <v>7</v>
+      </c>
+      <c r="D113" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="114" spans="1:3">
-      <c r="A114" s="2">
+      <c r="E113" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
         <v>113</v>
       </c>
-      <c r="B114" s="2" t="s">
+      <c r="B114" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C114" s="4" t="s">
+      <c r="C114" s="1">
+        <v>8</v>
+      </c>
+      <c r="D114" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="115" spans="1:3">
-      <c r="A115" s="2">
+      <c r="E114" s="5"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
         <v>114</v>
       </c>
-      <c r="B115" s="2" t="s">
+      <c r="B115" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C115" s="1">
+        <v>9</v>
+      </c>
+      <c r="D115" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="116" spans="1:3">
-      <c r="A116" s="2">
+      <c r="E115" s="7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
         <v>115</v>
       </c>
-      <c r="B116" s="2" t="s">
+      <c r="B116" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C116" s="1">
+        <v>10</v>
+      </c>
+      <c r="D116" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="117" spans="1:3">
-      <c r="A117" s="2">
+      <c r="E116" s="5"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
         <v>116</v>
       </c>
-      <c r="B117" s="2" t="s">
+      <c r="B117" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C117" s="1">
+        <v>11</v>
+      </c>
+      <c r="D117" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="118" spans="1:3">
-      <c r="A118" s="2">
+      <c r="E117" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
         <v>117</v>
       </c>
-      <c r="B118" s="2" t="s">
+      <c r="B118" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C118" s="4" t="s">
+      <c r="C118" s="1">
+        <v>12</v>
+      </c>
+      <c r="D118" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="119" spans="1:3">
-      <c r="A119" s="2">
+      <c r="E118" s="7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
         <v>118</v>
       </c>
-      <c r="B119" s="2" t="s">
+      <c r="B119" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C119" s="4" t="s">
+      <c r="C119" s="1">
+        <v>13</v>
+      </c>
+      <c r="D119" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="120" spans="1:3">
-      <c r="A120" s="2">
+      <c r="E119" s="5"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
         <v>119</v>
       </c>
-      <c r="B120" s="2" t="s">
+      <c r="B120" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C120" s="4" t="s">
+      <c r="C120" s="1">
+        <v>14</v>
+      </c>
+      <c r="D120" s="7" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="121" spans="1:3">
-      <c r="A121" s="2">
+      <c r="E120" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
         <v>120</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="B121" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C121" s="4" t="s">
+      <c r="C121" s="1">
+        <v>15</v>
+      </c>
+      <c r="D121" s="2" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="122" spans="1:3">
-      <c r="A122" s="2">
+      <c r="E121" s="5"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
         <v>121</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B122" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C122" s="4" t="s">
+      <c r="C122" s="1">
+        <v>1</v>
+      </c>
+      <c r="D122" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" s="2">
+      <c r="E122" s="5"/>
+      <c r="F122" s="9"/>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
         <v>122</v>
       </c>
-      <c r="B123" s="2" t="s">
+      <c r="B123" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C123" s="1">
+        <v>2</v>
+      </c>
+      <c r="D123" s="2" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="124" spans="1:3">
-      <c r="A124" s="2">
+      <c r="E123" s="5"/>
+      <c r="F123" s="9"/>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
         <v>123</v>
       </c>
-      <c r="B124" s="2" t="s">
+      <c r="B124" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C124" s="1">
+        <v>3</v>
+      </c>
+      <c r="D124" s="7" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="125" spans="1:3">
-      <c r="A125" s="2">
+      <c r="E124" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F124" s="9"/>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
         <v>124</v>
       </c>
-      <c r="B125" s="2" t="s">
+      <c r="B125" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C125" s="4" t="s">
+      <c r="C125" s="1">
+        <v>4</v>
+      </c>
+      <c r="D125" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="126" spans="1:3">
-      <c r="A126" s="2">
+      <c r="E125" s="5"/>
+      <c r="F125" s="9"/>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
         <v>125</v>
       </c>
-      <c r="B126" s="2" t="s">
+      <c r="B126" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C126" s="4" t="s">
+      <c r="C126" s="1">
+        <v>5</v>
+      </c>
+      <c r="D126" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="127" spans="1:3">
-      <c r="A127" s="2">
+      <c r="E126" s="5"/>
+      <c r="F126" s="9"/>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
         <v>126</v>
       </c>
-      <c r="B127" s="2" t="s">
+      <c r="B127" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C127" s="4" t="s">
+      <c r="C127" s="1">
+        <v>6</v>
+      </c>
+      <c r="D127" s="7" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="128" spans="1:3">
-      <c r="A128" s="2">
+      <c r="E127" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="F127" s="9"/>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" s="1">
         <v>127</v>
       </c>
-      <c r="B128" s="2" t="s">
+      <c r="B128" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C128" s="4" t="s">
+      <c r="C128" s="1">
+        <v>7</v>
+      </c>
+      <c r="D128" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="129" spans="1:3">
-      <c r="A129" s="2">
+      <c r="E128" s="5"/>
+      <c r="F128" s="9"/>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
         <v>128</v>
       </c>
-      <c r="B129" s="2" t="s">
+      <c r="B129" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C129" s="4" t="s">
+      <c r="C129" s="1">
+        <v>8</v>
+      </c>
+      <c r="D129" s="7" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="130" spans="1:3">
-      <c r="A130" s="2">
+      <c r="E129" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F129" s="9"/>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
         <v>129</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C130" s="4" t="s">
+      <c r="C130" s="1">
+        <v>9</v>
+      </c>
+      <c r="D130" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" s="2">
+      <c r="E130" s="5"/>
+      <c r="F130" s="9"/>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
         <v>130</v>
       </c>
-      <c r="B131" s="2" t="s">
+      <c r="B131" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C131" s="4" t="s">
+      <c r="C131" s="1">
+        <v>10</v>
+      </c>
+      <c r="D131" s="7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" s="2">
+      <c r="E131" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F131" s="9"/>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
         <v>131</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B132" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C132" s="4" t="s">
+      <c r="C132" s="1">
+        <v>11</v>
+      </c>
+      <c r="D132" s="7" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="2">
+      <c r="E132" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="F132" s="9"/>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
         <v>132</v>
       </c>
-      <c r="B133" s="2" t="s">
+      <c r="B133" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C133" s="4" t="s">
+      <c r="C133" s="1">
+        <v>12</v>
+      </c>
+      <c r="D133" s="7" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" s="2">
+      <c r="E133" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F133" s="9"/>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
         <v>133</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B134" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C134" s="4" t="s">
+      <c r="C134" s="1">
+        <v>13</v>
+      </c>
+      <c r="D134" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" s="2">
+      <c r="E134" s="2"/>
+      <c r="F134" s="9"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
         <v>134</v>
       </c>
-      <c r="B135" s="2" t="s">
+      <c r="B135" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C135" s="4" t="s">
+      <c r="C135" s="1">
+        <v>14</v>
+      </c>
+      <c r="D135" s="2" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="136" spans="1:3">
-      <c r="A136" s="2">
+      <c r="E135" s="2"/>
+      <c r="F135" s="9"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
         <v>135</v>
       </c>
-      <c r="B136" s="2" t="s">
+      <c r="B136" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C136" s="4" t="s">
+      <c r="C136" s="1">
+        <v>15</v>
+      </c>
+      <c r="D136" s="7" t="s">
         <v>146</v>
       </c>
+      <c r="E136" s="7" t="s">
+        <v>199</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <autoFilter ref="A1:E136" xr:uid="{DEDE1B6D-1479-42CC-A67D-1530C449213C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implementacion pagina introduccion, mejoras estabilidad y refactorizacion panel admin
</commit_message>
<xml_diff>
--- a/public/NUEVO TEST DE ENEAGRAMA COMPLETO.xlsx
+++ b/public/NUEVO TEST DE ENEAGRAMA COMPLETO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\App Test Eneagrama\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9C5D2A-6D4E-4ECA-96CF-2EC02C5F0394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B640358-125E-4ADF-A5B6-F8A53B15CA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{32DE2995-2421-4BC0-8390-3482C1C7896A}"/>
   </bookViews>
@@ -693,7 +693,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -709,12 +709,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -784,7 +778,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1125,6 +1119,7 @@
   <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
+    <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="90.69921875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="110.59765625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2096,10 +2091,10 @@
       <c r="A62" s="1">
         <v>61</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C62" s="1">
+      <c r="C62" s="11">
         <v>1</v>
       </c>
       <c r="D62" s="7" t="s">
@@ -2337,10 +2332,10 @@
       <c r="A77" s="1">
         <v>76</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C77" s="1">
+      <c r="C77" s="11">
         <v>1</v>
       </c>
       <c r="D77" s="2" t="s">
@@ -2806,10 +2801,10 @@
       <c r="A107" s="1">
         <v>106</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C107" s="1">
+      <c r="C107" s="11">
         <v>1</v>
       </c>
       <c r="D107" s="7" t="s">

</xml_diff>